<commit_message>
Add Sol monotributo invoice 23-jul for June service to Pelesson.
Registers factura $4.900.000 (CUIT 23-14614689-9) as PENDIENTE and
updates the UDESA reserve consolidation to separate billed vs collected.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,12 +46,8 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00666666"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -70,12 +66,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -115,11 +116,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,11 +131,15 @@
     <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -504,15 +507,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -525,387 +529,470 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobros extracto MP · retiros lista Sol cruzados con Dinero retirado Chris · armado 2026-07-23</t>
+          <t>Facturación SOL · cobros extracto MP · retiros Chris · act. 2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1) INGRESOS — facturado / cobrado LDO Pelesson</t>
+          <t>0) FACTURACIÓN monotributo Sol → LDO Pelesson</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Fecha factura</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Mes</t>
+          <t>Período</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>OpID</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>CUIT</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Monto ARS</t>
+          <t>Importe ARS</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Comentario</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Junio 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Aldo Pelesson / LDO Pelesson</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>23-14614689-9</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Servicio junio · factura 23/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Total facturado</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="9" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="10" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>1) COBROS MP — LDO Pelesson (históricos / sin factura asociada)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>OpID</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Monto ARS</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
         <v>46157</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Mayo</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>158620980755</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E11" s="13" t="n">
         <v>5000000</v>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Facturado/cobrado monotributo</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Cobro MP histórico</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
         <v>46185</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>163006931853</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E12" s="13" t="n">
         <v>4750000</v>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Facturado/cobrado monotributo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Total ingresos</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="10" t="n">
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Cobro MP histórico</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Total cobrado</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="15" t="n">
         <v>9750000</v>
       </c>
-      <c r="F9" s="9" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="F13" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>2) RETIROS a descontar</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Mes</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Fecha MP</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Mes Sol</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>OpID</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Monto ARS</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
+    <row r="17">
+      <c r="A17" s="16" t="n">
         <v>46183</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>163418872656</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E13" s="13" t="n">
+      <c r="E17" s="18" t="n">
         <v>500000</v>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>Retiro Junio (lista Sol)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="n">
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Retiro jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n">
         <v>46193</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>165013974648</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E14" s="13" t="n">
+      <c r="E18" s="18" t="n">
         <v>20000</v>
       </c>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>Lista=Julio; extracto=20-jun</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+    <row r="19">
+      <c r="A19" s="16" t="n">
         <v>46196</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>165530199038</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n">
+      <c r="E19" s="18" t="n">
         <v>150000</v>
       </c>
-      <c r="F15" s="12" t="inlineStr">
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>Lista=Julio; extracto=23-jun</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="11" t="n">
+    <row r="20">
+      <c r="A20" s="16" t="n">
         <v>46198</v>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>165824407784</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E20" s="18" t="n">
         <v>170100</v>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Lista=170000; extracto prevalece 170100</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Lista=170000; extracto=170100</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Total retiros (extracto)</t>
         </is>
       </c>
-      <c r="B17" s="9" t="n"/>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="10" t="n">
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="15" t="n">
         <v>840100</v>
       </c>
-      <c r="F17" s="9" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="F21" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>3) RESULTADO</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>(+) Total facturado / cobrado LDO Pelesson</t>
-        </is>
-      </c>
-      <c r="E20" s="14" t="n">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>(+) Total cobrado LDO Pelesson (extracto)</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="n">
         <v>9750000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>(−) Retiros (extracto)</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>840100</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>(=) SALDO RESERVA UDESA</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="17" t="n">
-        <v>8909900</v>
-      </c>
-      <c r="F22" s="16" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>Alternativa con montos redondeados de la lista (170.000):</t>
-        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Saldo lista (9.750.000 − 840.000)</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="n">
-        <v>8910000</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>Notas</t>
-        </is>
-      </c>
+          <t>(−) Retiros (extracto)</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>840100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>(=) SALDO RESERVA UDESA (caja)</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="22" t="n">
+        <v>8909900</v>
+      </c>
+      <c r="F26" s="21" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• Prevalece extracto oficial MP sobre texto de chat (fecha y monto 170.100).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>• Ruteo a reserva MP Chris: 16-may +5.000.000; 12-jun +4.500.000 (del cobro 4.750.000). Diff no reservada: 250.000.</t>
-        </is>
+          <t>Facturado pendiente de cobro (factura 23-jul servicio junio)</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>4900000</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>• No suma a matriz 2026 ni Almacén. Reserva aparte / MP No Gasto (Dinero reservado/retirado).</t>
+      <c r="A30" s="23" t="inlineStr">
+        <is>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>• Espejos: consolidacion_reserva_udesa.csv · CONSOLIDACION_RESERVA_UDESA.md</t>
+          <t>• Factura 23/7 $4.900.000 = registro facturación; aún PENDIENTE (no aumenta saldo caja hasta cobro en extracto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>• Cobros mayo/junio Pelesson siguen en caja de la reserva; no matchean 1:1 con la factura nueva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>• Registro canónico facturas: SOL/Facturacion_Monotributo_SOL_2026.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>• Prevalece extracto oficial MP sobre texto de chat (fecha y monto 170.100).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
+  <mergeCells count="6">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -917,16 +1004,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -969,53 +1056,48 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INGRESO</t>
-        </is>
-      </c>
-      <c r="B2" s="20" t="n">
-        <v>46157</v>
+          <t>FACTURA</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="n">
+        <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mayo</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>158620980755</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
-        </is>
-      </c>
-      <c r="F2" s="14" t="n">
-        <v>5000000</v>
+          <t>Factura monotributo Sol · Aldo Pelesson CUIT 23-14614689-9</t>
+        </is>
+      </c>
+      <c r="F2" s="19" t="n">
+        <v>4900000</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Facturado/cobrado monotributo LDO Pelesson</t>
+          <t>Servicio junio 2026 · PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INGRESO</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="n">
-        <v>46185</v>
+          <t>COBRO</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="n">
+        <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>163006931853</t>
+          <t>158620980755</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1023,23 +1105,23 @@
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F3" s="14" t="n">
-        <v>4750000</v>
+      <c r="F3" s="19" t="n">
+        <v>5000000</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Facturado/cobrado monotributo LDO Pelesson</t>
+          <t>Cobro MP histórico</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B4" s="20" t="n">
-        <v>46183</v>
+          <t>COBRO</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1048,20 +1130,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>163418872656</t>
+          <t>163006931853</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>500000</v>
+          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="n">
+        <v>4750000</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Retiro indicado Junio</t>
+          <t>Cobro MP histórico</t>
         </is>
       </c>
     </row>
@@ -1071,17 +1153,17 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B5" s="20" t="n">
-        <v>46193</v>
+      <c r="B5" s="24" t="n">
+        <v>46183</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>165013974648</t>
+          <t>163418872656</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1089,12 +1171,12 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F5" s="14" t="n">
-        <v>20000</v>
+      <c r="F5" s="19" t="n">
+        <v>500000</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lista Sol dijo Julio; extracto = 20-jun</t>
+          <t>Retiro Junio</t>
         </is>
       </c>
     </row>
@@ -1104,8 +1186,8 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
-        <v>46196</v>
+      <c r="B6" s="24" t="n">
+        <v>46193</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1114,7 +1196,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>165530199038</t>
+          <t>165013974648</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1122,12 +1204,12 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F6" s="14" t="n">
-        <v>150000</v>
+      <c r="F6" s="19" t="n">
+        <v>20000</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lista Sol dijo Julio; extracto = 23-jun</t>
+          <t>Lista Julio; extracto 20-jun</t>
         </is>
       </c>
     </row>
@@ -1137,8 +1219,8 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B7" s="20" t="n">
-        <v>46198</v>
+      <c r="B7" s="24" t="n">
+        <v>46196</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1147,7 +1229,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>165824407784</t>
+          <t>165530199038</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1155,67 +1237,142 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F7" s="14" t="n">
-        <v>170100</v>
+      <c r="F7" s="19" t="n">
+        <v>150000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lista Sol 170000; extracto prevalece 170100</t>
+          <t>Lista Julio; extracto 23-jun</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TOTAL_INGRESOS</t>
-        </is>
-      </c>
-      <c r="B8" s="20" t="n"/>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>165824407784</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Total facturado/cobrado LDO Pelesson</t>
-        </is>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>9750000</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>170100</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Lista 170000; extracto 170100</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TOTAL_RETIROS</t>
-        </is>
-      </c>
-      <c r="B9" s="20" t="n"/>
+          <t>TOTAL_FACTURADO</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Total retiros (extracto)</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>840100</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Total facturado monotributo</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SALDO</t>
-        </is>
-      </c>
-      <c r="B10" s="20" t="n"/>
+          <t>TOTAL_COBRADO</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Saldo Reserva UDESA</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="n">
+          <t>Total cobrado extracto</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>9750000</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TOTAL_RETIROS</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="n"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Total retiros extracto</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>840100</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SALDO_CAJA</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Saldo Reserva UDESA caja</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="n">
         <v>8909900</v>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>9750000 - 840100</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>9750000-840100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PENDIENTE_COBRO</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="n"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Facturas pendientes de cobro</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Factura 23-jul</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use 170000 for the Chris withdrawal in UDESA consolidation.
Keeps the retiro at Sol's stated amount and refreshes saldo to 8.910.000.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -515,7 +515,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -529,7 +529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Facturación SOL · cobros extracto MP · retiros Chris · act. 2026-07-23</t>
+          <t>Facturación SOL · cobros extracto MP · retiros Chris · act. 2026-07-23 · retiro 170.000</t>
         </is>
       </c>
     </row>
@@ -877,25 +877,25 @@
         </is>
       </c>
       <c r="E20" s="18" t="n">
-        <v>170100</v>
+        <v>170000</v>
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>Lista=170000; extracto=170100</t>
+          <t>Consolidado a 170000 (indicación Sol)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Total retiros (extracto)</t>
+          <t>Total retiros</t>
         </is>
       </c>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="15" t="n">
-        <v>840100</v>
+        <v>840000</v>
       </c>
       <c r="F21" s="6" t="n"/>
     </row>
@@ -919,11 +919,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>(−) Retiros (extracto)</t>
+          <t>(−) Retiros</t>
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>840100</v>
+        <v>840000</v>
       </c>
     </row>
     <row r="26">
@@ -936,7 +936,7 @@
       <c r="C26" s="21" t="n"/>
       <c r="D26" s="21" t="n"/>
       <c r="E26" s="22" t="n">
-        <v>8909900</v>
+        <v>8910000</v>
       </c>
       <c r="F26" s="21" t="n"/>
     </row>
@@ -974,14 +974,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>• Registro canónico facturas: SOL/Facturacion_Monotributo_SOL_2026.xlsx</t>
+          <t>• Retiro consolidado en $170.000 por indicación de Sol.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>• Prevalece extracto oficial MP sobre texto de chat (fecha y monto 170.100).</t>
+          <t>• Registro canónico facturas: SOL/Facturacion_Monotributo_SOL_2026.xlsx</t>
         </is>
       </c>
     </row>
@@ -1271,11 +1271,11 @@
         </is>
       </c>
       <c r="F8" s="19" t="n">
-        <v>170100</v>
+        <v>170000</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Lista 170000; extracto 170100</t>
+          <t>Consolidado a 170000 (indicación Sol)</t>
         </is>
       </c>
     </row>
@@ -1326,11 +1326,11 @@
       <c r="B11" s="24" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Total retiros extracto</t>
+          <t>Total retiros</t>
         </is>
       </c>
       <c r="F11" s="19" t="n">
-        <v>840100</v>
+        <v>840000</v>
       </c>
       <c r="G11" t="inlineStr"/>
     </row>
@@ -1347,11 +1347,11 @@
         </is>
       </c>
       <c r="F12" s="19" t="n">
-        <v>8909900</v>
+        <v>8910000</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>9750000-840100</t>
+          <t>9750000-840000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Load official Factura C 00001-00000027 into Sol monotributo.
Stores the ARCA PDF and refreshes billing fields (CAE, period, client,
concepto) plus UDESA consolidation references.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -116,24 +115,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,7 +140,11 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +539,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>0) FACTURACIÓN monotributo Sol → LDO Pelesson</t>
+          <t>0) FACTURACIÓN monotributo Sol → LDO Pelesson (Factura C 00001-00000027)</t>
         </is>
       </c>
     </row>
@@ -573,22 +576,22 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Comentario</t>
+          <t>Comp. / CAE / PDF</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="25" t="n">
         <v>46226</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Junio 2026</t>
+          <t>01/06–30/06/2026</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Aldo Pelesson / LDO Pelesson</t>
+          <t>PELESSON ALDO OSCAR</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -606,7 +609,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Servicio junio · factura 23/7</t>
+          <t>Factura C 00001-00000027 · CAE 86305115481677 · PDF SOL/_inbox/facturas_monotributo/27290390791_011_00001_00000027.pdf</t>
         </is>
       </c>
     </row>
@@ -665,7 +668,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="26" t="n">
         <v>46157</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -693,7 +696,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="26" t="n">
         <v>46185</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -774,7 +777,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="n">
+      <c r="A17" s="27" t="n">
         <v>46183</v>
       </c>
       <c r="B17" s="17" t="inlineStr">
@@ -802,7 +805,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="n">
+      <c r="A18" s="27" t="n">
         <v>46193</v>
       </c>
       <c r="B18" s="17" t="inlineStr">
@@ -830,7 +833,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="n">
+      <c r="A19" s="27" t="n">
         <v>46196</v>
       </c>
       <c r="B19" s="17" t="inlineStr">
@@ -858,7 +861,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="n">
+      <c r="A20" s="27" t="n">
         <v>46198</v>
       </c>
       <c r="B20" s="17" t="inlineStr">
@@ -943,7 +946,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Facturado pendiente de cobro (factura 23-jul servicio junio)</t>
+          <t>Facturado pendiente de cobro (Factura C 00001-00000027 · 23-jul · servicio junio)</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
@@ -960,7 +963,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>• Factura 23/7 $4.900.000 = registro facturación; aún PENDIENTE (no aumenta saldo caja hasta cobro en extracto).</t>
+          <t>• Factura C 00001-00000027 $4.900.000 = registro facturación (PDF ARCA); aún PENDIENTE (no aumenta saldo caja hasta cobro en extracto).</t>
         </is>
       </c>
     </row>
@@ -981,7 +984,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>• Registro canónico facturas: SOL/Facturacion_Monotributo_SOL_2026.xlsx</t>
+          <t>• Registro canónico: SOL/Facturacion_Monotributo_SOL_2026.xlsx · PDF en SOL/_inbox/facturas_monotributo/</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1062,7 @@
           <t>FACTURA</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="28" t="n">
         <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1067,9 +1070,14 @@
           <t>Junio</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>00001-00000027</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Factura monotributo Sol · Aldo Pelesson CUIT 23-14614689-9</t>
+          <t>Factura C monotributo Sol · PELESSON ALDO OSCAR CUIT 23-14614689-9</t>
         </is>
       </c>
       <c r="F2" s="19" t="n">
@@ -1077,7 +1085,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Servicio junio 2026 · PENDIENTE</t>
+          <t>Período 01/06-30/06/2026 · CAE 86305115481677 · PENDIENTE · PDF ARCA</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1095,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="28" t="n">
         <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1120,7 +1128,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="28" t="n">
         <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1153,7 +1161,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="28" t="n">
         <v>46183</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1186,7 +1194,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="28" t="n">
         <v>46193</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1219,7 +1227,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="28" t="n">
         <v>46196</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1252,7 +1260,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="28" t="n">
         <v>46198</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -1285,7 +1293,7 @@
           <t>TOTAL_FACTURADO</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n"/>
+      <c r="B9" s="28" t="n"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Total facturado monotributo</t>
@@ -1306,7 +1314,7 @@
           <t>TOTAL_COBRADO</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n"/>
+      <c r="B10" s="28" t="n"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Total cobrado extracto</t>
@@ -1315,7 +1323,6 @@
       <c r="F10" s="19" t="n">
         <v>9750000</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1323,7 +1330,7 @@
           <t>TOTAL_RETIROS</t>
         </is>
       </c>
-      <c r="B11" s="24" t="n"/>
+      <c r="B11" s="28" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Total retiros</t>
@@ -1332,7 +1339,6 @@
       <c r="F11" s="19" t="n">
         <v>840000</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1340,7 +1346,7 @@
           <t>SALDO_CAJA</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n"/>
+      <c r="B12" s="28" t="n"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Saldo Reserva UDESA caja</t>
@@ -1361,7 +1367,7 @@
           <t>PENDIENTE_COBRO</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n"/>
+      <c r="B13" s="28" t="n"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Facturas pendientes de cobro</t>

</xml_diff>

<commit_message>
Mark Factura C 00001-00000027 as paid via MP on 23-jul.
Updates Sol monotributo billing to COBRADO and refreshes UDESA
cash balance to 13.810.000; OpID awaits next MP extract.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -46,7 +47,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -60,7 +61,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E3F0"/>
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -70,22 +81,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,36 +111,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,15 +502,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -532,7 +524,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Facturación SOL · cobros extracto MP · retiros Chris · act. 2026-07-23 · retiro 170.000</t>
+          <t>Factura C 00001-00000027 COBRADA 23/07/2026 MP · saldo caja 13.810.000</t>
         </is>
       </c>
     </row>
@@ -576,12 +568,12 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Comp. / CAE / PDF</t>
+          <t>Comp. / CAE / cobro</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="n">
+      <c r="A6" s="5" t="n">
         <v>46226</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -604,12 +596,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>COBRADO</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Factura C 00001-00000027 · CAE 86305115481677 · PDF SOL/_inbox/facturas_monotributo/27290390791_011_00001_00000027.pdf</t>
+          <t>00001-00000027 · CAE 86305115481677 · cobro MP 23/07/2026</t>
         </is>
       </c>
     </row>
@@ -631,7 +623,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>1) COBROS MP — LDO Pelesson (históricos / sin factura asociada)</t>
+          <t>1) COBROS — LDO Pelesson</t>
         </is>
       </c>
     </row>
@@ -668,7 +660,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="n">
+      <c r="A11" s="11" t="n">
         <v>46157</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -696,7 +688,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="n">
+      <c r="A12" s="11" t="n">
         <v>46185</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -724,265 +716,293 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="11" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>(pendiente extracto)</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Cobro MP Factura C 00001-00000027</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Confirmación Sol · abonada hoy MP</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Total cobrado</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="15" t="n">
-        <v>9750000</v>
-      </c>
-      <c r="F13" s="6" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="16" t="n">
+        <v>14650000</v>
+      </c>
+      <c r="F14" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>2) RETIROS a descontar</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Fecha MP</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Mes Sol</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>OpID</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Monto ARS</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="27" t="n">
+    <row r="18">
+      <c r="A18" s="17" t="n">
         <v>46183</v>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>163418872656</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D18" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E18" s="19" t="n">
         <v>500000</v>
       </c>
-      <c r="F17" s="17" t="inlineStr">
+      <c r="F18" s="18" t="inlineStr">
         <is>
           <t>Retiro jun</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="27" t="n">
+    <row r="19">
+      <c r="A19" s="17" t="n">
         <v>46193</v>
       </c>
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C18" s="17" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>165013974648</t>
         </is>
       </c>
-      <c r="D18" s="17" t="inlineStr">
+      <c r="D19" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E19" s="19" t="n">
         <v>20000</v>
       </c>
-      <c r="F18" s="17" t="inlineStr">
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>Lista=Julio; extracto=20-jun</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="27" t="n">
+    <row r="20">
+      <c r="A20" s="17" t="n">
         <v>46196</v>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>165530199038</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D20" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E20" s="19" t="n">
         <v>150000</v>
       </c>
-      <c r="F19" s="17" t="inlineStr">
+      <c r="F20" s="18" t="inlineStr">
         <is>
           <t>Lista=Julio; extracto=23-jun</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="27" t="n">
+    <row r="21">
+      <c r="A21" s="17" t="n">
         <v>46198</v>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>165824407784</t>
         </is>
       </c>
-      <c r="D20" s="17" t="inlineStr">
+      <c r="D21" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E21" s="19" t="n">
         <v>170000</v>
       </c>
-      <c r="F20" s="17" t="inlineStr">
-        <is>
-          <t>Consolidado a 170000 (indicación Sol)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Consolidado a 170000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Total retiros</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="15" t="n">
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="16" t="n">
         <v>840000</v>
       </c>
-      <c r="F21" s="6" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="F22" s="15" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>3) RESULTADO</t>
         </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>(+) Total cobrado LDO Pelesson (extracto)</t>
-        </is>
-      </c>
-      <c r="E24" s="19" t="n">
-        <v>9750000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>(+) Total cobrado LDO Pelesson</t>
+        </is>
+      </c>
+      <c r="E25" s="20" t="n">
+        <v>14650000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>(−) Retiros</t>
         </is>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E26" s="20" t="n">
         <v>840000</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="20" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>(=) SALDO RESERVA UDESA (caja)</t>
         </is>
       </c>
-      <c r="B26" s="21" t="n"/>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="22" t="n">
-        <v>8910000</v>
-      </c>
-      <c r="F26" s="21" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Facturado pendiente de cobro (Factura C 00001-00000027 · 23-jul · servicio junio)</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="n">
-        <v>4900000</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="23" t="inlineStr">
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="22" t="n">
+        <v>13810000</v>
+      </c>
+      <c r="F27" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Facturado pendiente de cobro</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>• Factura C 00001-00000027 $4.900.000 = registro facturación (PDF ARCA); aún PENDIENTE (no aumenta saldo caja hasta cobro en extracto).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>• Cobros mayo/junio Pelesson siguen en caja de la reserva; no matchean 1:1 con la factura nueva.</t>
+          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP (confirmación Sol).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>• Retiro consolidado en $170.000 por indicación de Sol.</t>
+          <t>• OpID del cobro 23-jul pendiente: el extracto MP en repo corta el 18-jul.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t>• Retiro consolidado en $170.000 por indicación de Sol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>• Registro canónico: SOL/Facturacion_Monotributo_SOL_2026.xlsx · PDF en SOL/_inbox/facturas_monotributo/</t>
         </is>
@@ -993,9 +1013,9 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1007,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1016,7 +1036,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1062,7 +1082,7 @@
           <t>FACTURA</t>
         </is>
       </c>
-      <c r="B2" s="28" t="n">
+      <c r="B2" s="24" t="n">
         <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1077,15 +1097,15 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Factura C monotributo Sol · PELESSON ALDO OSCAR CUIT 23-14614689-9</t>
-        </is>
-      </c>
-      <c r="F2" s="19" t="n">
+          <t>Factura C monotributo Sol · PELESSON ALDO OSCAR</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="n">
         <v>4900000</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Período 01/06-30/06/2026 · CAE 86305115481677 · PENDIENTE · PDF ARCA</t>
+          <t>COBRADO 23/07/2026 MP · CAE 86305115481677</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1115,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B3" s="28" t="n">
+      <c r="B3" s="24" t="n">
         <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1113,7 +1133,7 @@
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="20" t="n">
         <v>5000000</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -1128,7 +1148,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B4" s="28" t="n">
+      <c r="B4" s="24" t="n">
         <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1146,7 +1166,7 @@
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="20" t="n">
         <v>4750000</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -1158,33 +1178,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B5" s="28" t="n">
-        <v>46183</v>
+          <t>COBRO</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>46226</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>163418872656</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>500000</v>
+          <t>Cobro MP Factura C 00001-00000027</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>4900000</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Retiro Junio</t>
+          <t>Confirmación Sol · OpID pendiente extracto</t>
         </is>
       </c>
     </row>
@@ -1194,17 +1209,17 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B6" s="28" t="n">
-        <v>46193</v>
+      <c r="B6" s="24" t="n">
+        <v>46183</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>165013974648</t>
+          <t>163418872656</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1212,12 +1227,12 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F6" s="19" t="n">
-        <v>20000</v>
+      <c r="F6" s="20" t="n">
+        <v>500000</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lista Julio; extracto 20-jun</t>
+          <t>Retiro Junio</t>
         </is>
       </c>
     </row>
@@ -1227,8 +1242,8 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B7" s="28" t="n">
-        <v>46196</v>
+      <c r="B7" s="24" t="n">
+        <v>46193</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1237,7 +1252,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>165530199038</t>
+          <t>165013974648</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1245,12 +1260,12 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F7" s="19" t="n">
-        <v>150000</v>
+      <c r="F7" s="20" t="n">
+        <v>20000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lista Julio; extracto 23-jun</t>
+          <t>Lista Julio; extracto 20-jun</t>
         </is>
       </c>
     </row>
@@ -1260,8 +1275,8 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B8" s="28" t="n">
-        <v>46198</v>
+      <c r="B8" s="24" t="n">
+        <v>46196</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1270,7 +1285,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>165824407784</t>
+          <t>165530199038</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1278,109 +1293,140 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F8" s="19" t="n">
-        <v>170000</v>
+      <c r="F8" s="20" t="n">
+        <v>150000</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Consolidado a 170000 (indicación Sol)</t>
+          <t>Lista Julio; extracto 23-jun</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TOTAL_FACTURADO</t>
-        </is>
-      </c>
-      <c r="B9" s="28" t="n"/>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>165824407784</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Total facturado monotributo</t>
-        </is>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>4900000</v>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>170000</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>Consolidado a 170000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TOTAL_COBRADO</t>
-        </is>
-      </c>
-      <c r="B10" s="28" t="n"/>
+          <t>TOTAL_FACTURADO</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Total cobrado extracto</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="n">
-        <v>9750000</v>
+          <t>Total facturado monotributo</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>COBRADO</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TOTAL_RETIROS</t>
-        </is>
-      </c>
-      <c r="B11" s="28" t="n"/>
+          <t>TOTAL_COBRADO</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="n"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Total retiros</t>
-        </is>
-      </c>
-      <c r="F11" s="19" t="n">
-        <v>840000</v>
-      </c>
+          <t>Total cobrado</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>14650000</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SALDO_CAJA</t>
-        </is>
-      </c>
-      <c r="B12" s="28" t="n"/>
+          <t>TOTAL_RETIROS</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Saldo Reserva UDESA caja</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="n">
-        <v>8910000</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>9750000-840000</t>
-        </is>
-      </c>
+          <t>Total retiros</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>840000</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>SALDO_CAJA</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="n"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Saldo Reserva UDESA caja</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>13810000</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>14650000-840000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>PENDIENTE_COBRO</t>
         </is>
       </c>
-      <c r="B13" s="28" t="n"/>
-      <c r="E13" t="inlineStr">
+      <c r="B14" s="24" t="n"/>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Facturas pendientes de cobro</t>
         </is>
       </c>
-      <c r="F13" s="19" t="n">
-        <v>4900000</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Factura 23-jul</t>
-        </is>
-      </c>
+      <c r="F14" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Route 23-jul Pelesson cobro to Reserva Chris / UDESA.
Records Dinero reservado Chris for the $4.900.000 invoice payment
and keeps OpID pending the next MP extract.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -47,7 +47,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E5F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -111,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +137,9 @@
     <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -502,10 +510,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
@@ -517,21 +525,21 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Consolidación Reserva UDESA — monotributo LDO Pelesson</t>
+          <t>Consolidación Reserva UDESA / Chris — monotributo LDO Pelesson</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Factura C 00001-00000027 COBRADA 23/07/2026 MP · saldo caja 13.810.000</t>
+          <t>Cobro factura 00001-00000027 → Reserva Chris · saldo 13.810.000</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>0) FACTURACIÓN monotributo Sol → LDO Pelesson (Factura C 00001-00000027)</t>
+          <t>0) FACTURACIÓN → destino Reserva Chris</t>
         </is>
       </c>
     </row>
@@ -568,7 +576,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Comp. / CAE / cobro</t>
+          <t>Destino</t>
         </is>
       </c>
     </row>
@@ -601,7 +609,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>00001-00000027 · CAE 86305115481677 · cobro MP 23/07/2026</t>
+          <t>Reserva Chris · Factura C 00001-00000027 · CAE 86305115481677</t>
         </is>
       </c>
     </row>
@@ -739,7 +747,7 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Confirmación Sol · abonada hoy MP</t>
+          <t>→ Reserva Chris (confirmación Sol)</t>
         </is>
       </c>
     </row>
@@ -760,19 +768,19 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2) RETIROS a descontar</t>
+          <t>1b) RUTEO a Reserva Chris (Dinero reservado Chris)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Fecha MP</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Mes Sol</t>
+          <t>Mes</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -798,224 +806,362 @@
     </row>
     <row r="18">
       <c r="A18" s="17" t="n">
-        <v>46183</v>
+        <v>46158</v>
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>163418872656</t>
+          <t>158758469069</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
+          <t>Dinero reservado Chris</t>
         </is>
       </c>
       <c r="E18" s="19" t="n">
-        <v>500000</v>
+        <v>5000000</v>
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Retiro jun</t>
+          <t>Cobro Pelesson 15-may</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="n">
-        <v>46193</v>
+        <v>46185</v>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Julio*</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>165013974648</t>
+          <t>163024353651</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
+          <t>Dinero reservado Chris</t>
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>20000</v>
+        <v>4500000</v>
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Lista=Julio; extracto=20-jun</t>
+          <t>Parcial cobro 4.750.000</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>(pendiente extracto)</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>Dinero reservado Chris</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>Confirmación Sol: factura → Reserva Chris</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Total ruteado a Chris (Pelesson/factura)</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="16" t="n">
+        <v>14400000</v>
+      </c>
+      <c r="F21" s="15" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2) RETIROS (Dinero retirado Chris)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Fecha MP</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Mes Sol</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>OpID</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Monto ARS</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>163418872656</t>
+        </is>
+      </c>
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
+        <is>
+          <t>Retiro jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>Julio*</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>165013974648</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>Lista=Julio; extracto=20-jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="n">
         <v>46196</v>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C27" s="21" t="inlineStr">
         <is>
           <t>165530199038</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E27" s="22" t="n">
         <v>150000</v>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F27" s="21" t="inlineStr">
         <is>
           <t>Lista=Julio; extracto=23-jun</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="17" t="n">
+    <row r="28">
+      <c r="A28" s="20" t="n">
         <v>46198</v>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>165824407784</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E28" s="22" t="n">
         <v>170000</v>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F28" s="21" t="inlineStr">
         <is>
           <t>Consolidado a 170000</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Total retiros</t>
         </is>
       </c>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="16" t="n">
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="16" t="n">
         <v>840000</v>
       </c>
-      <c r="F22" s="15" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>3) RESULTADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>(+) Total cobrado LDO Pelesson</t>
-        </is>
-      </c>
-      <c r="E25" s="20" t="n">
-        <v>14650000</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>(−) Retiros</t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="n">
-        <v>840000</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>(=) SALDO RESERVA UDESA (caja)</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="22" t="n">
-        <v>13810000</v>
-      </c>
-      <c r="F27" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Facturado pendiente de cobro</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="F29" s="15" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="inlineStr">
-        <is>
-          <t>Notas</t>
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>3) RESULTADO Reserva Chris / UDESA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP (confirmación Sol).</t>
-        </is>
+          <t>(+) Total cobrado LDO Pelesson</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="n">
+        <v>14650000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>• OpID del cobro 23-jul pendiente: el extracto MP en repo corta el 18-jul.</t>
-        </is>
+          <t>(−) Retiros Chris</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="n">
+        <v>840000</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>(=) SALDO RESERVA UDESA / CHRIS</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="25" t="n">
+        <v>13810000</v>
+      </c>
+      <c r="F34" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Facturado pendiente de cobro</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP → Reserva Chris (confirmación Sol).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>• OpID del cobro/reserva 23-jul pendiente: el extracto MP en repo corta el 18-jul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>• Retiro consolidado en $170.000 por indicación de Sol.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>• Registro canónico: SOL/Facturacion_Monotributo_SOL_2026.xlsx · PDF en SOL/_inbox/facturas_monotributo/</t>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>• UDESA = reserva MP etiquetada Chris (Dinero reservado / retirado Chris).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1027,7 +1173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1036,7 +1182,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1082,7 +1228,7 @@
           <t>FACTURA</t>
         </is>
       </c>
-      <c r="B2" s="24" t="n">
+      <c r="B2" s="27" t="n">
         <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1100,12 +1246,12 @@
           <t>Factura C monotributo Sol · PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F2" s="20" t="n">
+      <c r="F2" s="23" t="n">
         <v>4900000</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>COBRADO 23/07/2026 MP · CAE 86305115481677</t>
+          <t>COBRADO → Reserva Chris</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1261,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B3" s="24" t="n">
+      <c r="B3" s="27" t="n">
         <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1133,7 +1279,7 @@
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F3" s="20" t="n">
+      <c r="F3" s="23" t="n">
         <v>5000000</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -1148,7 +1294,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="27" t="n">
         <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1166,7 +1312,7 @@
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F4" s="20" t="n">
+      <c r="F4" s="23" t="n">
         <v>4750000</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -1181,7 +1327,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="27" t="n">
         <v>46226</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1194,111 +1340,106 @@
           <t>Cobro MP Factura C 00001-00000027</t>
         </is>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="23" t="n">
         <v>4900000</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Confirmación Sol · OpID pendiente extracto</t>
+          <t>→ Reserva Chris · OpID pendiente</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>46183</v>
+          <t>RESERVA</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="n">
+        <v>46158</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Mayo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>163418872656</t>
+          <t>158758469069</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="n">
-        <v>500000</v>
+          <t>Dinero reservado Chris</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>5000000</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Retiro Junio</t>
+          <t>Ruteo cobro 15-may</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B7" s="24" t="n">
-        <v>46193</v>
+          <t>RESERVA</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>46185</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>165013974648</t>
+          <t>163024353651</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>20000</v>
+          <t>Dinero reservado Chris</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>4500000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lista Julio; extracto 20-jun</t>
+          <t>Ruteo parcial cobro 12-jun</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="n">
-        <v>46196</v>
+          <t>RESERVA</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="n">
+        <v>46226</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>165530199038</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="n">
-        <v>150000</v>
+          <t>Dinero reservado Chris</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>4900000</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Lista Julio; extracto 23-jun</t>
+          <t>Confirmación Sol · factura → Chris</t>
         </is>
       </c>
     </row>
@@ -1308,17 +1449,17 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
-        <v>46198</v>
+      <c r="B9" s="27" t="n">
+        <v>46183</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>165824407784</t>
+          <t>163418872656</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1326,69 +1467,113 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F9" s="20" t="n">
-        <v>170000</v>
+      <c r="F9" s="23" t="n">
+        <v>500000</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Consolidado a 170000</t>
+          <t>Retiro Junio</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TOTAL_FACTURADO</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="n"/>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B10" s="27" t="n">
+        <v>46193</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>165013974648</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Total facturado monotributo</t>
-        </is>
-      </c>
-      <c r="F10" s="20" t="n">
-        <v>4900000</v>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>20000</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>COBRADO</t>
+          <t>Lista Julio; extracto 20-jun</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TOTAL_COBRADO</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="n"/>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="n">
+        <v>46196</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>165530199038</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Total cobrado</t>
-        </is>
-      </c>
-      <c r="F11" s="20" t="n">
-        <v>14650000</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="n">
+        <v>150000</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Lista Julio; extracto 23-jun</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TOTAL_RETIROS</t>
-        </is>
-      </c>
-      <c r="B12" s="24" t="n"/>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>165824407784</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Total retiros</t>
-        </is>
-      </c>
-      <c r="F12" s="20" t="n">
-        <v>840000</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="n">
+        <v>170000</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Consolidado a 170000</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1396,13 +1581,13 @@
           <t>SALDO_CAJA</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n"/>
+      <c r="B13" s="27" t="n"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Saldo Reserva UDESA caja</t>
-        </is>
-      </c>
-      <c r="F13" s="20" t="n">
+          <t>Saldo Reserva UDESA / Chris</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="n">
         <v>13810000</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -1410,23 +1595,6 @@
           <t>14650000-840000</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>PENDIENTE_COBRO</t>
-        </is>
-      </c>
-      <c r="B14" s="24" t="n"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Facturas pendientes de cobro</t>
-        </is>
-      </c>
-      <c r="F14" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Chris reserve top-up to match UDESA cash balance.
With Chris at 10.300.000 and UDESA target 13.810.000, records
3.510.000 to restore into Dinero reservado Chris.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -116,35 +116,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -532,7 +544,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cobro factura 00001-00000027 → Reserva Chris · saldo 13.810.000</t>
+          <t>Chris actual $10.300.000 · UDESA $13.810.000 · a reponer $3.510.000</t>
         </is>
       </c>
     </row>
@@ -581,7 +593,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="28" t="n">
         <v>46226</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -668,7 +680,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="29" t="n">
         <v>46157</v>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -696,7 +708,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="29" t="n">
         <v>46185</v>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -724,7 +736,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="29" t="n">
         <v>46226</v>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -805,7 +817,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="n">
+      <c r="A18" s="30" t="n">
         <v>46158</v>
       </c>
       <c r="B18" s="18" t="inlineStr">
@@ -833,7 +845,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="n">
+      <c r="A19" s="30" t="n">
         <v>46185</v>
       </c>
       <c r="B19" s="18" t="inlineStr">
@@ -861,7 +873,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="n">
+      <c r="A20" s="30" t="n">
         <v>46226</v>
       </c>
       <c r="B20" s="18" t="inlineStr">
@@ -942,7 +954,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="n">
+      <c r="A25" s="31" t="n">
         <v>46183</v>
       </c>
       <c r="B25" s="21" t="inlineStr">
@@ -970,7 +982,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="n">
+      <c r="A26" s="31" t="n">
         <v>46193</v>
       </c>
       <c r="B26" s="21" t="inlineStr">
@@ -998,7 +1010,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="n">
+      <c r="A27" s="31" t="n">
         <v>46196</v>
       </c>
       <c r="B27" s="21" t="inlineStr">
@@ -1026,7 +1038,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="n">
+      <c r="A28" s="31" t="n">
         <v>46198</v>
       </c>
       <c r="B28" s="21" t="inlineStr">
@@ -1119,32 +1131,45 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="26" t="inlineStr">
-        <is>
-          <t>Notas</t>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>4) REPOSICIÓN a Reserva Chris (para igualar saldo caja UDESA)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP → Reserva Chris (confirmación Sol).</t>
-        </is>
+          <t>Saldo caja UDESA consolidado (cobrado − retiros)</t>
+        </is>
+      </c>
+      <c r="E39" s="32" t="n">
+        <v>13810000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>• OpID del cobro/reserva 23-jul pendiente: el extracto MP en repo corta el 18-jul.</t>
-        </is>
+          <t>Saldo actual Reserva Chris (MP)</t>
+        </is>
+      </c>
+      <c r="E40" s="33" t="n">
+        <v>10300000</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>• Retiro consolidado en $170.000 por indicación de Sol.</t>
-        </is>
-      </c>
+      <c r="A41" s="34" t="inlineStr">
+        <is>
+          <t>(=) A DEVOLVER / REPONER a Reserva Chris</t>
+        </is>
+      </c>
+      <c r="B41" s="21" t="n"/>
+      <c r="C41" s="21" t="n"/>
+      <c r="D41" s="21" t="n"/>
+      <c r="E41" s="35" t="n">
+        <v>3510000</v>
+      </c>
+      <c r="F41" s="21" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1153,12 +1178,55 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>• Para alinear Reserva Chris con saldo UDESA: reservar $3.510.000 a Dinero reservado Chris.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP → Reserva Chris (confirmación Sol).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>• OpID del cobro/reserva 23-jul pendiente: el extracto MP en repo corta el 18-jul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>• Retiro consolidado en $170.000 por indicación de Sol.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>• UDESA = reserva MP etiquetada Chris (Dinero reservado / retirado Chris).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A23:G23"/>
@@ -1173,7 +1241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1228,7 +1296,7 @@
           <t>FACTURA</t>
         </is>
       </c>
-      <c r="B2" s="27" t="n">
+      <c r="B2" s="36" t="n">
         <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1261,7 +1329,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B3" s="27" t="n">
+      <c r="B3" s="36" t="n">
         <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1294,7 +1362,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="36" t="n">
         <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1327,7 +1395,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n">
+      <c r="B5" s="36" t="n">
         <v>46226</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1355,7 +1423,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="36" t="n">
         <v>46158</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1388,7 +1456,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="36" t="n">
         <v>46185</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1421,7 +1489,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="36" t="n">
         <v>46226</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -1449,7 +1517,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="36" t="n">
         <v>46183</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -1482,7 +1550,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
+      <c r="B10" s="36" t="n">
         <v>46193</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -1515,7 +1583,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="36" t="n">
         <v>46196</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -1548,7 +1616,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
+      <c r="B12" s="36" t="n">
         <v>46198</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -1581,7 +1649,7 @@
           <t>SALDO_CAJA</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n"/>
+      <c r="B13" s="36" t="n"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Saldo Reserva UDESA / Chris</t>
@@ -1593,6 +1661,63 @@
       <c r="G13" t="inlineStr">
         <is>
           <t>14650000-840000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SALDO_CHRIS_ACTUAL</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Saldo actual Reserva Chris (MP)</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="n">
+        <v>10300000</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Indicación Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>A_REPONER_CHRIS</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="n"/>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>A devolver/reponer a Reserva Chris</t>
+        </is>
+      </c>
+      <c r="F15" s="39" t="n">
+        <v>3510000</v>
+      </c>
+      <c r="G15" s="37" t="inlineStr">
+        <is>
+          <t>13810000 - 10300000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 3.510.000 debt owed to Reserva Chris / UDESA.
Marks the gap vs the 10.300.000 Chris balance as deuda pendiente
de devolver a Dinero reservado Chris.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -544,7 +543,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Chris actual $10.300.000 · UDESA $13.810.000 · a reponer $3.510.000</t>
+          <t>Chris actual $10.300.000 · UDESA $13.810.000 · DEUDA con la reserva $3.510.000</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1132,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>4) REPOSICIÓN a Reserva Chris (para igualar saldo caja UDESA)</t>
+          <t>4) DEUDA con la Reserva Chris / UDESA</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1159,7 @@
     <row r="41">
       <c r="A41" s="34" t="inlineStr">
         <is>
-          <t>(=) A DEVOLVER / REPONER a Reserva Chris</t>
+          <t>(=) DEUDA CON LA RESERVA (le debo)</t>
         </is>
       </c>
       <c r="B41" s="21" t="n"/>
@@ -1188,7 +1187,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>• Para alinear Reserva Chris con saldo UDESA: reservar $3.510.000 a Dinero reservado Chris.</t>
+          <t>• Sol le debe $3.510.000 a Reserva Chris / UDESA. Para saldar: Dinero reservado Chris por ese monto.</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1694,7 @@
     <row r="15">
       <c r="A15" s="37" t="inlineStr">
         <is>
-          <t>A_REPONER_CHRIS</t>
+          <t>DEUDA_RESERVA_CHRIS</t>
         </is>
       </c>
       <c r="B15" s="38" t="n">
@@ -1709,7 +1708,7 @@
       <c r="D15" s="37" t="n"/>
       <c r="E15" s="37" t="inlineStr">
         <is>
-          <t>A devolver/reponer a Reserva Chris</t>
+          <t>Deuda con Reserva Chris / UDESA (le debo)</t>
         </is>
       </c>
       <c r="F15" s="39" t="n">
@@ -1717,7 +1716,7 @@
       </c>
       <c r="G15" s="37" t="inlineStr">
         <is>
-          <t>13810000 - 10300000</t>
+          <t>13810000 - 10300000 · pendiente de devolver</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record 2.000.000 payment toward Chris/UDESA reserve debt.
Updates Chris balance to 12.300.000 and remaining debt to 1.510.000.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -115,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,6 +157,9 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -521,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -543,7 +547,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Chris actual $10.300.000 · UDESA $13.810.000 · DEUDA con la reserva $3.510.000</t>
+          <t>Pago 25-jul $2.000.000 a Chris · deuda restante $1.510.000 · UDESA $13.810.000</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1153,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Saldo actual Reserva Chris (MP)</t>
+          <t>Saldo Reserva Chris al 23/07</t>
         </is>
       </c>
       <c r="E40" s="33" t="n">
@@ -1159,7 +1163,7 @@
     <row r="41">
       <c r="A41" s="34" t="inlineStr">
         <is>
-          <t>(=) DEUDA CON LA RESERVA (le debo)</t>
+          <t>Deuda inicial (le debía)</t>
         </is>
       </c>
       <c r="B41" s="21" t="n"/>
@@ -1171,25 +1175,38 @@
       <c r="F41" s="21" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>• UDESA = reserva MP etiquetada Chris (Dinero reservado / retirado Chris).</t>
-        </is>
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>(−) Pago a la reserva 25/07/2026</t>
+        </is>
+      </c>
+      <c r="E42" s="13" t="n">
+        <v>2000000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="26" t="inlineStr">
         <is>
-          <t>Notas</t>
-        </is>
+          <t>Saldo actual Reserva Chris</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>12300000</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>• Sol le debe $3.510.000 a Reserva Chris / UDESA. Para saldar: Dinero reservado Chris por ese monto.</t>
-        </is>
-      </c>
+      <c r="A44" s="34" t="inlineStr">
+        <is>
+          <t>(=) DEUDA RESTANTE (le debo)</t>
+        </is>
+      </c>
+      <c r="B44" s="21" t="n"/>
+      <c r="C44" s="21" t="n"/>
+      <c r="D44" s="21" t="n"/>
+      <c r="E44" s="35" t="n">
+        <v>1510000</v>
+      </c>
+      <c r="F44" s="21" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1199,26 +1216,44 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>• OpID del cobro/reserva 23-jul pendiente: el extracto MP en repo corta el 18-jul.</t>
+      <c r="A46" s="26" t="inlineStr">
+        <is>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>• Retiro consolidado en $170.000 por indicación de Sol.</t>
+          <t>• 25/07/2026: Sol pagó $2.000.000 a Reserva Chris. Deuda restante $1.510.000.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP → Reserva Chris.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>• OpIDs de cobro/reserva 23-jul y pago 25-jul pendientes de próximo extracto MP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>• UDESA = reserva MP etiquetada Chris (Dinero reservado / retirado Chris).</t>
         </is>
       </c>
     </row>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
@@ -1240,7 +1275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1664,59 +1699,116 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="40" t="inlineStr">
+        <is>
+          <t>PAGO_DEUDA</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="n">
+        <v>46228</v>
+      </c>
+      <c r="C14" s="40" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D14" s="40" t="n"/>
+      <c r="E14" s="40" t="inlineStr">
+        <is>
+          <t>Pago a Reserva Chris (devolución parcial deuda)</t>
+        </is>
+      </c>
+      <c r="F14" s="42" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="G14" s="40" t="inlineStr">
+        <is>
+          <t>Confirmación Sol · OpID pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SALDO_CHRIS_ANTES</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Saldo Reserva Chris antes del pago 25-jul</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="n">
+        <v>10300000</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Indicación Sol 23/07</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>SALDO_CHRIS_ACTUAL</t>
         </is>
       </c>
-      <c r="B14" s="36" t="n">
-        <v>46226</v>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B16" s="36" t="n">
+        <v>46228</v>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Saldo actual Reserva Chris (MP)</t>
         </is>
       </c>
-      <c r="F14" s="23" t="n">
-        <v>10300000</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Indicación Sol</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="37" t="inlineStr">
+      <c r="F16" s="23" t="n">
+        <v>12300000</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>10300000 + 2000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="inlineStr">
         <is>
           <t>DEUDA_RESERVA_CHRIS</t>
         </is>
       </c>
-      <c r="B15" s="38" t="n">
-        <v>46226</v>
-      </c>
-      <c r="C15" s="37" t="inlineStr">
+      <c r="B17" s="38" t="n">
+        <v>46228</v>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="D15" s="37" t="n"/>
-      <c r="E15" s="37" t="inlineStr">
-        <is>
-          <t>Deuda con Reserva Chris / UDESA (le debo)</t>
-        </is>
-      </c>
-      <c r="F15" s="39" t="n">
-        <v>3510000</v>
-      </c>
-      <c r="G15" s="37" t="inlineStr">
-        <is>
-          <t>13810000 - 10300000 · pendiente de devolver</t>
+      <c r="D17" s="37" t="n"/>
+      <c r="E17" s="37" t="inlineStr">
+        <is>
+          <t>Deuda restante con Reserva Chris / UDESA (le debo)</t>
+        </is>
+      </c>
+      <c r="F17" s="39" t="n">
+        <v>1510000</v>
+      </c>
+      <c r="G17" s="37" t="inlineStr">
+        <is>
+          <t>3510000 - 2000000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh UDESA Excel after Chris 500.000 reserve withdrawal.
Rebuilds the workbook so the 25-jul retiro and 11.800.000
Chris balance match the consolidation CSV/MD.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -116,50 +116,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -525,15 +513,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -547,7 +535,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pago 25-jul $2.000.000 a Chris · deuda restante $1.510.000 · UDESA $13.810.000</t>
+          <t>Retiro Chris 25-jul $500.000 · reserva $11.800.000 · deuda $1.510.000 · UDESA $13.310.000</t>
         </is>
       </c>
     </row>
@@ -596,7 +584,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="n">
+      <c r="A6" s="5" t="n">
         <v>46226</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -624,468 +612,495 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Reserva Chris · Factura C 00001-00000027 · CAE 86305115481677</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Total facturado</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="10" t="n">
+          <t>Reserva Chris · Factura C 00001-00000027</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>1) COBROS — LDO Pelesson</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>OpID</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Monto ARS</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Mayo</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>158620980755</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Cobro MP histórico</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>163006931853</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>4750000</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Cobro MP histórico</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>(pendiente extracto)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Cobro MP Factura C 00001-00000027</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="n">
         <v>4900000</v>
       </c>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>1) COBROS — LDO Pelesson</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>→ Reserva Chris</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Total cobrado</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="13" t="n">
+        <v>14650000</v>
+      </c>
+      <c r="F13" s="12" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>1b) ENTRADAS a Reserva Chris</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>OpID</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Monto ARS</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="29" t="n">
-        <v>46157</v>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="14" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>Mayo</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>158620980755</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>158758469069</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Dinero reservado Chris</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="n">
         <v>5000000</v>
       </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>Cobro MP histórico</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="29" t="n">
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>Cobro Pelesson 15-may</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
         <v>46185</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>163006931853</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>4750000</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>Cobro MP histórico</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="29" t="n">
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>163024353651</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Dinero reservado Chris</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>Parcial cobro 4.750.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="n">
         <v>46226</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>(pendiente extracto)</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Cobro MP Factura C 00001-00000027</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="n">
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Dinero reservado Chris</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="n">
         <v>4900000</v>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>→ Reserva Chris (confirmación Sol)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Total cobrado</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="n"/>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="15" t="n"/>
-      <c r="E14" s="16" t="n">
-        <v>14650000</v>
-      </c>
-      <c r="F14" s="15" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>1b) RUTEO a Reserva Chris (Dinero reservado Chris)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Mes</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>Factura → Reserva Chris</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>(pendiente extracto)</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Pago / reposición parcial deuda</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Confirmación Sol</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2) RETIROS (Dinero retirado Chris)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Fecha MP</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Mes Sol</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>OpID</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Monto ARS</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="30" t="n">
-        <v>46158</v>
-      </c>
-      <c r="B18" s="18" t="inlineStr">
-        <is>
-          <t>Mayo</t>
-        </is>
-      </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>158758469069</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Dinero reservado Chris</t>
-        </is>
-      </c>
-      <c r="E18" s="19" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>Cobro Pelesson 15-may</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="30" t="n">
-        <v>46185</v>
-      </c>
-      <c r="B19" s="18" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
-        <is>
-          <t>163024353651</t>
-        </is>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t>Dinero reservado Chris</t>
-        </is>
-      </c>
-      <c r="E19" s="19" t="n">
-        <v>4500000</v>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>Parcial cobro 4.750.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="30" t="n">
-        <v>46226</v>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>163418872656</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>Retiro jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>46193</v>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Julio*</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>165013974648</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>extracto=20-jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Julio*</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>165530199038</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>extracto=23-jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Julio*</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>165824407784</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>170000</v>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>consolidado 170000</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>(pendiente extracto)</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>Dinero reservado Chris</t>
-        </is>
-      </c>
-      <c r="E20" s="19" t="n">
-        <v>4900000</v>
-      </c>
-      <c r="F20" s="18" t="inlineStr">
-        <is>
-          <t>Confirmación Sol: factura → Reserva Chris</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>Total ruteado a Chris (Pelesson/factura)</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="n"/>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="16" t="n">
-        <v>14400000</v>
-      </c>
-      <c r="F21" s="15" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>2) RETIROS (Dinero retirado Chris)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Fecha MP</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Mes Sol</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>OpID</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Monto ARS</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Nota</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="31" t="n">
-        <v>46183</v>
-      </c>
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>163418872656</t>
-        </is>
-      </c>
-      <c r="D25" s="21" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E25" s="22" t="n">
+      <c r="E28" s="19" t="n">
         <v>500000</v>
       </c>
-      <c r="F25" s="21" t="inlineStr">
-        <is>
-          <t>Retiro jun</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="31" t="n">
-        <v>46193</v>
-      </c>
-      <c r="B26" s="21" t="inlineStr">
-        <is>
-          <t>Julio*</t>
-        </is>
-      </c>
-      <c r="C26" s="21" t="inlineStr">
-        <is>
-          <t>165013974648</t>
-        </is>
-      </c>
-      <c r="D26" s="21" t="inlineStr">
-        <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="E26" s="22" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F26" s="21" t="inlineStr">
-        <is>
-          <t>Lista=Julio; extracto=20-jun</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="31" t="n">
-        <v>46196</v>
-      </c>
-      <c r="B27" s="21" t="inlineStr">
-        <is>
-          <t>Julio*</t>
-        </is>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>165530199038</t>
-        </is>
-      </c>
-      <c r="D27" s="21" t="inlineStr">
-        <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="E27" s="22" t="n">
-        <v>150000</v>
-      </c>
-      <c r="F27" s="21" t="inlineStr">
-        <is>
-          <t>Lista=Julio; extracto=23-jun</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="31" t="n">
-        <v>46198</v>
-      </c>
-      <c r="B28" s="21" t="inlineStr">
-        <is>
-          <t>Julio*</t>
-        </is>
-      </c>
-      <c r="C28" s="21" t="inlineStr">
-        <is>
-          <t>165824407784</t>
-        </is>
-      </c>
-      <c r="D28" s="21" t="inlineStr">
-        <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="E28" s="22" t="n">
-        <v>170000</v>
-      </c>
-      <c r="F28" s="21" t="inlineStr">
-        <is>
-          <t>Consolidado a 170000</t>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>Bajar reserva · Sol</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>Total retiros</t>
         </is>
       </c>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="16" t="n">
-        <v>840000</v>
-      </c>
-      <c r="F29" s="15" t="n"/>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="13" t="n">
+        <v>1340000</v>
+      </c>
+      <c r="F29" s="12" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>3) RESULTADO Reserva Chris / UDESA</t>
+          <t>3) RESULTADO</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1110,7 @@
           <t>(+) Total cobrado LDO Pelesson</t>
         </is>
       </c>
-      <c r="E32" s="23" t="n">
+      <c r="E32" s="20" t="n">
         <v>14650000</v>
       </c>
     </row>
@@ -1105,165 +1120,133 @@
           <t>(−) Retiros Chris</t>
         </is>
       </c>
-      <c r="E33" s="23" t="n">
-        <v>840000</v>
+      <c r="E33" s="20" t="n">
+        <v>1340000</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>(=) SALDO RESERVA UDESA / CHRIS</t>
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>(=) SALDO CAJA UDESA consolidado</t>
         </is>
       </c>
       <c r="B34" s="6" t="n"/>
       <c r="C34" s="6" t="n"/>
       <c r="D34" s="6" t="n"/>
-      <c r="E34" s="25" t="n">
-        <v>13810000</v>
+      <c r="E34" s="22" t="n">
+        <v>13310000</v>
       </c>
       <c r="F34" s="6" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Facturado pendiente de cobro</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="n">
-        <v>0</v>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>4) DEUDA con la Reserva Chris / UDESA</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Saldo caja UDESA consolidado</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>13310000</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>4) DEUDA con la Reserva Chris / UDESA</t>
-        </is>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Saldo Reserva Chris al 23/07</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="n">
+        <v>10300000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Saldo caja UDESA consolidado (cobrado − retiros)</t>
-        </is>
-      </c>
-      <c r="E39" s="32" t="n">
-        <v>13810000</v>
+          <t>(+) Pago a la reserva 25/07</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="n">
+        <v>2000000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Saldo Reserva Chris al 23/07</t>
-        </is>
-      </c>
-      <c r="E40" s="33" t="n">
-        <v>10300000</v>
+          <t>(−) Retiro Chris 25/07 (bajar reserva)</t>
+        </is>
+      </c>
+      <c r="E40" s="19" t="n">
+        <v>500000</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="34" t="inlineStr">
-        <is>
-          <t>Deuda inicial (le debía)</t>
-        </is>
-      </c>
-      <c r="B41" s="21" t="n"/>
-      <c r="C41" s="21" t="n"/>
-      <c r="D41" s="21" t="n"/>
-      <c r="E41" s="35" t="n">
-        <v>3510000</v>
-      </c>
-      <c r="F41" s="21" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Saldo actual Reserva Chris</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>11800000</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="26" t="inlineStr">
-        <is>
-          <t>(−) Pago a la reserva 25/07/2026</t>
-        </is>
-      </c>
-      <c r="E42" s="13" t="n">
-        <v>2000000</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="26" t="inlineStr">
-        <is>
-          <t>Saldo actual Reserva Chris</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="n">
-        <v>12300000</v>
-      </c>
+      <c r="A42" s="24" t="inlineStr">
+        <is>
+          <t>(=) DEUDA RESTANTE (le debo)</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="25" t="n">
+        <v>1510000</v>
+      </c>
+      <c r="F42" s="18" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="34" t="inlineStr">
-        <is>
-          <t>(=) DEUDA RESTANTE (le debo)</t>
-        </is>
-      </c>
-      <c r="B44" s="21" t="n"/>
-      <c r="C44" s="21" t="n"/>
-      <c r="D44" s="21" t="n"/>
-      <c r="E44" s="35" t="n">
-        <v>1510000</v>
-      </c>
-      <c r="F44" s="21" t="n"/>
+      <c r="A44" s="26" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP → Reserva Chris (confirmación Sol).</t>
+          <t>• 25/07: retiro Chris $500.000 (bajar reserva). Reserva actual $11.800.000.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="26" t="inlineStr">
-        <is>
-          <t>Notas</t>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>• 25/07: pago previo $2.000.000. Deuda restante $1.510.000.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>• 25/07/2026: Sol pagó $2.000.000 a Reserva Chris. Deuda restante $1.510.000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>• Factura C 00001-00000027 $4.900.000 COBRADA 23/07/2026 con MP → Reserva Chris.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>• OpIDs de cobro/reserva 23-jul y pago 25-jul pendientes de próximo extracto MP.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>• UDESA = reserva MP etiquetada Chris (Dinero reservado / retirado Chris).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
+          <t>• OpIDs 23/25-jul pendientes de próximo extracto MP.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A8:G8"/>
     <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A38:G38"/>
-    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1284,7 +1267,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1330,7 +1313,7 @@
           <t>FACTURA</t>
         </is>
       </c>
-      <c r="B2" s="36" t="n">
+      <c r="B2" s="27" t="n">
         <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1348,7 +1331,7 @@
           <t>Factura C monotributo Sol · PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F2" s="23" t="n">
+      <c r="F2" s="20" t="n">
         <v>4900000</v>
       </c>
       <c r="G2" t="inlineStr">
@@ -1363,7 +1346,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B3" s="36" t="n">
+      <c r="B3" s="27" t="n">
         <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1381,7 +1364,7 @@
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F3" s="23" t="n">
+      <c r="F3" s="20" t="n">
         <v>5000000</v>
       </c>
       <c r="G3" t="inlineStr">
@@ -1396,7 +1379,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B4" s="36" t="n">
+      <c r="B4" s="27" t="n">
         <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1414,7 +1397,7 @@
           <t>Transferencia recibida PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="F4" s="23" t="n">
+      <c r="F4" s="20" t="n">
         <v>4750000</v>
       </c>
       <c r="G4" t="inlineStr">
@@ -1429,7 +1412,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B5" s="36" t="n">
+      <c r="B5" s="27" t="n">
         <v>46226</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1442,12 +1425,12 @@
           <t>Cobro MP Factura C 00001-00000027</t>
         </is>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="20" t="n">
         <v>4900000</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>→ Reserva Chris · OpID pendiente</t>
+          <t>→ Reserva Chris</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1440,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B6" s="36" t="n">
+      <c r="B6" s="27" t="n">
         <v>46158</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1475,7 +1458,7 @@
           <t>Dinero reservado Chris</t>
         </is>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="20" t="n">
         <v>5000000</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -1490,7 +1473,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B7" s="36" t="n">
+      <c r="B7" s="27" t="n">
         <v>46185</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1508,12 +1491,12 @@
           <t>Dinero reservado Chris</t>
         </is>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="20" t="n">
         <v>4500000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Ruteo parcial cobro 12-jun</t>
+          <t>Ruteo parcial 12-jun</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1506,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B8" s="36" t="n">
+      <c r="B8" s="27" t="n">
         <v>46226</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -1536,45 +1519,40 @@
           <t>Dinero reservado Chris</t>
         </is>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="20" t="n">
         <v>4900000</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Confirmación Sol · factura → Chris</t>
+          <t>Factura → Chris</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="n">
-        <v>46183</v>
+          <t>PAGO_DEUDA</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="n">
+        <v>46228</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>163418872656</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="F9" s="23" t="n">
-        <v>500000</v>
+          <t>Pago a Reserva Chris</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>2000000</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Retiro Junio</t>
+          <t>Confirmación Sol</t>
         </is>
       </c>
     </row>
@@ -1584,17 +1562,17 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B10" s="36" t="n">
-        <v>46193</v>
+      <c r="B10" s="27" t="n">
+        <v>46183</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>165013974648</t>
+          <t>163418872656</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1602,12 +1580,12 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F10" s="23" t="n">
-        <v>20000</v>
+      <c r="F10" s="20" t="n">
+        <v>500000</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Lista Julio; extracto 20-jun</t>
+          <t>Retiro Junio</t>
         </is>
       </c>
     </row>
@@ -1617,8 +1595,8 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B11" s="36" t="n">
-        <v>46196</v>
+      <c r="B11" s="27" t="n">
+        <v>46193</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1627,7 +1605,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>165530199038</t>
+          <t>165013974648</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1635,12 +1613,12 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F11" s="23" t="n">
-        <v>150000</v>
+      <c r="F11" s="20" t="n">
+        <v>20000</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Lista Julio; extracto 23-jun</t>
+          <t>extracto 20-jun</t>
         </is>
       </c>
     </row>
@@ -1650,8 +1628,8 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B12" s="36" t="n">
-        <v>46198</v>
+      <c r="B12" s="27" t="n">
+        <v>46196</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1660,7 +1638,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>165824407784</t>
+          <t>165530199038</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1668,90 +1646,94 @@
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="F12" s="23" t="n">
-        <v>170000</v>
+      <c r="F12" s="20" t="n">
+        <v>150000</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Consolidado a 170000</t>
+          <t>extracto 23-jun</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SALDO_CAJA</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="n"/>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>165824407784</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Saldo Reserva UDESA / Chris</t>
-        </is>
-      </c>
-      <c r="F13" s="23" t="n">
-        <v>13810000</v>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="n">
+        <v>170000</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>14650000-840000</t>
+          <t>consolidado 170000</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="40" t="inlineStr">
-        <is>
-          <t>PAGO_DEUDA</t>
-        </is>
-      </c>
-      <c r="B14" s="41" t="n">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="n">
         <v>46228</v>
       </c>
-      <c r="C14" s="40" t="inlineStr">
+      <c r="C14" s="28" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="D14" s="40" t="n"/>
-      <c r="E14" s="40" t="inlineStr">
-        <is>
-          <t>Pago a Reserva Chris (devolución parcial deuda)</t>
-        </is>
-      </c>
-      <c r="F14" s="42" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="G14" s="40" t="inlineStr">
-        <is>
-          <t>Confirmación Sol · OpID pendiente</t>
+      <c r="D14" s="28" t="n"/>
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>Dinero retirado Chris</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>Bajar reserva · Sol</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SALDO_CHRIS_ANTES</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="n">
-        <v>46226</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Julio</t>
+          <t>SALDO_CAJA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Saldo Reserva Chris antes del pago 25-jul</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="n">
-        <v>10300000</v>
+          <t>Saldo caja UDESA consolidado</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>13310000</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Indicación Sol 23/07</t>
+          <t>14650000-1340000</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1743,7 @@
           <t>SALDO_CHRIS_ACTUAL</t>
         </is>
       </c>
-      <c r="B16" s="36" t="n">
+      <c r="B16" s="27" t="n">
         <v>46228</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1771,44 +1753,44 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Saldo actual Reserva Chris (MP)</t>
-        </is>
-      </c>
-      <c r="F16" s="23" t="n">
-        <v>12300000</v>
+          <t>Saldo actual Reserva Chris</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="n">
+        <v>11800000</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10300000 + 2000000</t>
+          <t>10300000+2000000-500000</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="37" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>DEUDA_RESERVA_CHRIS</t>
         </is>
       </c>
-      <c r="B17" s="38" t="n">
+      <c r="B17" s="29" t="n">
         <v>46228</v>
       </c>
-      <c r="C17" s="37" t="inlineStr">
+      <c r="C17" s="28" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="D17" s="37" t="n"/>
-      <c r="E17" s="37" t="inlineStr">
-        <is>
-          <t>Deuda restante con Reserva Chris / UDESA (le debo)</t>
-        </is>
-      </c>
-      <c r="F17" s="39" t="n">
+      <c r="D17" s="28" t="n"/>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>Deuda restante (le debo)</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="n">
         <v>1510000</v>
       </c>
-      <c r="G17" s="37" t="inlineStr">
-        <is>
-          <t>3510000 - 2000000</t>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>13310000-11800000</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Set Sol-to-Chris debt as 3.510.000 minus 2.000.000 paid.
Remaining debt today is 1.510.000 after Sol's reserve payment.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -116,25 +116,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,10 +144,16 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,7 +541,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Retiro Chris 25-jul $500.000 · reserva $11.800.000 · deuda $1.510.000 · UDESA $13.310.000</t>
+          <t>Deuda original 3.510.000 − pago 2.000.000 = deuda hoy 1.510.000 · Chris $11.800.000</t>
         </is>
       </c>
     </row>
@@ -584,7 +590,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="31" t="n">
         <v>46226</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -656,7 +662,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="32" t="n">
         <v>46157</v>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -684,7 +690,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="32" t="n">
         <v>46185</v>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -712,7 +718,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="32" t="n">
         <v>46226</v>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -793,7 +799,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="n">
+      <c r="A17" s="33" t="n">
         <v>46158</v>
       </c>
       <c r="B17" s="15" t="inlineStr">
@@ -821,7 +827,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="n">
+      <c r="A18" s="33" t="n">
         <v>46185</v>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -849,7 +855,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="n">
+      <c r="A19" s="33" t="n">
         <v>46226</v>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -877,7 +883,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="n">
+      <c r="A20" s="33" t="n">
         <v>46228</v>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -944,7 +950,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="34" t="n">
         <v>46183</v>
       </c>
       <c r="B24" s="18" t="inlineStr">
@@ -972,7 +978,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="n">
+      <c r="A25" s="34" t="n">
         <v>46193</v>
       </c>
       <c r="B25" s="18" t="inlineStr">
@@ -1000,7 +1006,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="n">
+      <c r="A26" s="34" t="n">
         <v>46196</v>
       </c>
       <c r="B26" s="18" t="inlineStr">
@@ -1028,7 +1034,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="n">
+      <c r="A27" s="34" t="n">
         <v>46198</v>
       </c>
       <c r="B27" s="18" t="inlineStr">
@@ -1056,7 +1062,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="17" t="n">
+      <c r="A28" s="34" t="n">
         <v>46228</v>
       </c>
       <c r="B28" s="18" t="inlineStr">
@@ -1141,72 +1147,70 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>4) DEUDA con la Reserva Chris / UDESA</t>
+          <t>4) DEUDA Sol → Reserva Chris</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Saldo caja UDESA consolidado</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>13310000</v>
+          <t>Deuda original</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="n">
+        <v>3510000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Saldo Reserva Chris al 23/07</t>
-        </is>
-      </c>
-      <c r="E38" s="23" t="n">
-        <v>10300000</v>
+          <t>(−) Pago Sol a la reserva 25/07</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="n">
+        <v>2000000</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>(+) Pago a la reserva 25/07</t>
-        </is>
-      </c>
-      <c r="E39" s="10" t="n">
-        <v>2000000</v>
-      </c>
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>(=) SALDO DEUDA A HOY</t>
+        </is>
+      </c>
+      <c r="B39" s="18" t="n"/>
+      <c r="C39" s="18" t="n"/>
+      <c r="D39" s="18" t="n"/>
+      <c r="E39" s="25" t="n">
+        <v>1510000</v>
+      </c>
+      <c r="F39" s="18" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>(−) Retiro Chris 25/07 (bajar reserva)</t>
-        </is>
-      </c>
-      <c r="E40" s="19" t="n">
-        <v>500000</v>
+          <t>Saldo actual Reserva Chris (caja)</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>11800000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Saldo actual Reserva Chris</t>
+          <t>(ref) Retiro Chris 25/07 bajar reserva</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>11800000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>(=) DEUDA RESTANTE (le debo)</t>
-        </is>
-      </c>
+      <c r="A42" s="24" t="n"/>
       <c r="B42" s="18" t="n"/>
       <c r="C42" s="18" t="n"/>
       <c r="D42" s="18" t="n"/>
-      <c r="E42" s="25" t="n">
-        <v>1510000</v>
-      </c>
+      <c r="E42" s="25" t="n"/>
       <c r="F42" s="18" t="n"/>
     </row>
     <row r="44">
@@ -1219,14 +1223,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>• 25/07: retiro Chris $500.000 (bajar reserva). Reserva actual $11.800.000.</t>
+          <t>• Deuda original $3.510.000 − pago Sol $2.000.000 = deuda hoy $1.510.000.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>• 25/07: pago previo $2.000.000. Deuda restante $1.510.000.</t>
+          <t>• 25/07 retiro Chris $500.000 (baja reserva). Chris actual $11.800.000.</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1313,7 +1317,7 @@
           <t>FACTURA</t>
         </is>
       </c>
-      <c r="B2" s="27" t="n">
+      <c r="B2" s="35" t="n">
         <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1346,7 +1350,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B3" s="27" t="n">
+      <c r="B3" s="35" t="n">
         <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1379,7 +1383,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="35" t="n">
         <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1412,7 +1416,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n">
+      <c r="B5" s="35" t="n">
         <v>46226</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1440,7 +1444,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="35" t="n">
         <v>46158</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1473,7 +1477,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="35" t="n">
         <v>46185</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1506,7 +1510,7 @@
           <t>RESERVA</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="35" t="n">
         <v>46226</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -1534,7 +1538,7 @@
           <t>PAGO_DEUDA</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="35" t="n">
         <v>46228</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -1562,7 +1566,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
+      <c r="B10" s="35" t="n">
         <v>46183</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -1595,7 +1599,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="35" t="n">
         <v>46193</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -1628,7 +1632,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B12" s="27" t="n">
+      <c r="B12" s="35" t="n">
         <v>46196</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -1661,7 +1665,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B13" s="27" t="n">
+      <c r="B13" s="35" t="n">
         <v>46198</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -1694,7 +1698,7 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B14" s="29" t="n">
+      <c r="B14" s="36" t="n">
         <v>46228</v>
       </c>
       <c r="C14" s="28" t="inlineStr">
@@ -1743,7 +1747,7 @@
           <t>SALDO_CHRIS_ACTUAL</t>
         </is>
       </c>
-      <c r="B16" s="27" t="n">
+      <c r="B16" s="35" t="n">
         <v>46228</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -1771,7 +1775,7 @@
           <t>DEUDA_RESERVA_CHRIS</t>
         </is>
       </c>
-      <c r="B17" s="29" t="n">
+      <c r="B17" s="36" t="n">
         <v>46228</v>
       </c>
       <c r="C17" s="28" t="inlineStr">
@@ -1782,7 +1786,7 @@
       <c r="D17" s="28" t="n"/>
       <c r="E17" s="28" t="inlineStr">
         <is>
-          <t>Deuda restante (le debo)</t>
+          <t>Deuda restante Sol a Reserva Chris (le debo)</t>
         </is>
       </c>
       <c r="F17" s="30" t="n">
@@ -1790,7 +1794,35 @@
       </c>
       <c r="G17" s="28" t="inlineStr">
         <is>
-          <t>13310000-11800000</t>
+          <t>3510000 - 2000000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DEUDA_INICIAL</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Deuda original Sol a Reserva Chris</t>
+        </is>
+      </c>
+      <c r="F18" s="20" t="n">
+        <v>3510000</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Indicación Sol</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync UDESA Excel after clearing the 1.510.000 Chris debt.
Workbook now shows debt fully paid and Chris cash at 13.310.000.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
+++ b/CIUDAD/_inbox/Consolidacion_Reserva_UDESA.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -116,44 +116,39 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -522,13 +517,13 @@
   <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -541,21 +536,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Deuda original 3.510.000 − pago 2.000.000 = deuda hoy 1.510.000 · Chris $11.800.000</t>
+          <t>Deuda SALDADA · pagos 2.000.000 + 1.510.000 · Chris $13.310.000 = UDESA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>0) FACTURACIÓN → destino Reserva Chris</t>
+          <t>0) FACTURACIÓN → Reserva Chris</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Fecha factura</t>
+          <t>Fecha</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -575,7 +570,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Importe ARS</t>
+          <t>Importe</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -590,7 +585,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31" t="n">
+      <c r="A6" s="5" t="n">
         <v>46226</v>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -618,14 +613,14 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Reserva Chris · Factura C 00001-00000027</t>
+          <t>Reserva Chris · 00001-00000027</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>1) COBROS — LDO Pelesson</t>
+          <t>1) COBROS LDO Pelesson</t>
         </is>
       </c>
     </row>
@@ -652,7 +647,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Monto ARS</t>
+          <t>Monto</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -662,7 +657,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="n">
+      <c r="A10" s="8" t="n">
         <v>46157</v>
       </c>
       <c r="B10" s="9" t="inlineStr">
@@ -677,7 +672,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
+          <t>Transferencia recibida PELESSON</t>
         </is>
       </c>
       <c r="E10" s="10" t="n">
@@ -685,12 +680,12 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Cobro MP histórico</t>
+          <t>histórico</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="n">
+      <c r="A11" s="8" t="n">
         <v>46185</v>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -705,7 +700,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
+          <t>Transferencia recibida PELESSON</t>
         </is>
       </c>
       <c r="E11" s="10" t="n">
@@ -713,12 +708,12 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Cobro MP histórico</t>
+          <t>histórico</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="n">
+      <c r="A12" s="8" t="n">
         <v>46226</v>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -728,12 +723,12 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>(pendiente extracto)</t>
+          <t>(pendiente)</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Cobro MP Factura C 00001-00000027</t>
+          <t>Cobro Factura C 00001-00000027</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
@@ -741,7 +736,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>→ Reserva Chris</t>
+          <t>→ Chris</t>
         </is>
       </c>
     </row>
@@ -762,7 +757,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>1b) ENTRADAS a Reserva Chris</t>
+          <t>1b) ENTRADAS Reserva Chris</t>
         </is>
       </c>
     </row>
@@ -789,7 +784,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Monto ARS</t>
+          <t>Monto</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -799,7 +794,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="33" t="n">
+      <c r="A17" s="14" t="n">
         <v>46158</v>
       </c>
       <c r="B17" s="15" t="inlineStr">
@@ -822,12 +817,12 @@
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>Cobro Pelesson 15-may</t>
+          <t>cobro 15-may</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="33" t="n">
+      <c r="A18" s="14" t="n">
         <v>46185</v>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -850,12 +845,12 @@
       </c>
       <c r="F18" s="15" t="inlineStr">
         <is>
-          <t>Parcial cobro 4.750.000</t>
+          <t>parcial 4.75M</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="n">
+      <c r="A19" s="14" t="n">
         <v>46226</v>
       </c>
       <c r="B19" s="15" t="inlineStr">
@@ -865,7 +860,7 @@
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>(pendiente extracto)</t>
+          <t>(pendiente)</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
@@ -878,12 +873,12 @@
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>Factura → Reserva Chris</t>
+          <t>factura</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="33" t="n">
+      <c r="A20" s="14" t="n">
         <v>46228</v>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -893,12 +888,12 @@
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>(pendiente extracto)</t>
+          <t>(pendiente)</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Pago / reposición parcial deuda</t>
+          <t>Pago deuda Sol</t>
         </is>
       </c>
       <c r="E20" s="16" t="n">
@@ -906,315 +901,319 @@
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>Confirmación Sol</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>2) RETIROS (Dinero retirado Chris)</t>
+          <t>parcial</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>(pendiente)</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Pago deuda Sol</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>1510000</v>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>salda deuda</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Fecha MP</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Mes Sol</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2) RETIROS Chris</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>OpID</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Monto ARS</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="34" t="n">
+    <row r="25">
+      <c r="A25" s="17" t="n">
         <v>46183</v>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>163418872656</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D25" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E25" s="19" t="n">
         <v>500000</v>
       </c>
-      <c r="F24" s="18" t="inlineStr">
-        <is>
-          <t>Retiro jun</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="34" t="n">
+      <c r="F25" s="18" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n">
         <v>46193</v>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>165013974648</t>
         </is>
       </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="D26" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E26" s="19" t="n">
         <v>20000</v>
       </c>
-      <c r="F25" s="18" t="inlineStr">
-        <is>
-          <t>extracto=20-jun</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="34" t="n">
+      <c r="F26" s="18" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
         <v>46196</v>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>165530199038</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E26" s="19" t="n">
+      <c r="E27" s="19" t="n">
         <v>150000</v>
       </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>extracto=23-jun</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="34" t="n">
+      <c r="F27" s="18" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n">
         <v>46198</v>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Julio*</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>165824407784</t>
         </is>
       </c>
-      <c r="D27" s="18" t="inlineStr">
+      <c r="D28" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E27" s="19" t="n">
+      <c r="E28" s="19" t="n">
         <v>170000</v>
       </c>
-      <c r="F27" s="18" t="inlineStr">
-        <is>
-          <t>consolidado 170000</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="34" t="n">
+      <c r="F28" s="18" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
         <v>46228</v>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
-        <is>
-          <t>(pendiente extracto)</t>
-        </is>
-      </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>(pendiente)</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E29" s="19" t="n">
         <v>500000</v>
       </c>
-      <c r="F28" s="18" t="inlineStr">
-        <is>
-          <t>Bajar reserva · Sol</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>bajar reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>Total retiros</t>
         </is>
       </c>
-      <c r="B29" s="12" t="n"/>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="13" t="n">
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="13" t="n">
         <v>1340000</v>
       </c>
-      <c r="F29" s="12" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="F30" s="12" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>3) RESULTADO</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>(+) Total cobrado LDO Pelesson</t>
-        </is>
-      </c>
-      <c r="E32" s="20" t="n">
-        <v>14650000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>(+) Cobrado Pelesson</t>
+        </is>
+      </c>
+      <c r="E33" s="20" t="n">
+        <v>14650000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>(−) Retiros Chris</t>
         </is>
       </c>
-      <c r="E33" s="20" t="n">
+      <c r="E34" s="20" t="n">
         <v>1340000</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr">
-        <is>
-          <t>(=) SALDO CAJA UDESA consolidado</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="22" t="n">
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>(=) SALDO CAJA UDESA</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="22" t="n">
         <v>13310000</v>
       </c>
-      <c r="F34" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>4) DEUDA Sol → Reserva Chris</t>
-        </is>
-      </c>
+      <c r="F35" s="6" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Deuda original</t>
-        </is>
-      </c>
-      <c r="E37" s="23" t="n">
-        <v>3510000</v>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>4) DEUDA Sol → Chris</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>(−) Pago Sol a la reserva 25/07</t>
-        </is>
-      </c>
-      <c r="E38" s="10" t="n">
+          <t>Deuda original</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="n">
+        <v>3510000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>(−) Pago Sol 25/07</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="n">
         <v>2000000</v>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>(=) SALDO DEUDA A HOY</t>
-        </is>
-      </c>
-      <c r="B39" s="18" t="n"/>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="25" t="n">
-        <v>1510000</v>
-      </c>
-      <c r="F39" s="18" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Saldo actual Reserva Chris (caja)</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>11800000</v>
+          <t>(−) Pago Sol 27/07</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="n">
+        <v>1510000</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>(ref) Retiro Chris 25/07 bajar reserva</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>500000</v>
-      </c>
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>(=) SALDO DEUDA A HOY</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="6" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="n"/>
-      <c r="B42" s="18" t="n"/>
-      <c r="C42" s="18" t="n"/>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="25" t="n"/>
-      <c r="F42" s="18" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Saldo actual Reserva Chris</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>13310000</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="26" t="inlineStr">
+      <c r="A44" s="24" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -1223,34 +1222,34 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>• Deuda original $3.510.000 − pago Sol $2.000.000 = deuda hoy $1.510.000.</t>
+          <t>• Deuda $3.510.000 − $2.000.000 − $1.510.000 = $0 (SALDADA).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>• 25/07 retiro Chris $500.000 (baja reserva). Chris actual $11.800.000.</t>
+          <t>• Chris $13.310.000 alineada con saldo caja UDESA.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>• OpIDs 23/25-jul pendientes de próximo extracto MP.</t>
+          <t>• OpIDs 23/25/27-jul pendientes de próximo extracto MP.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A32:G32"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1262,16 +1261,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1317,7 +1316,7 @@
           <t>FACTURA</t>
         </is>
       </c>
-      <c r="B2" s="35" t="n">
+      <c r="B2" s="25" t="n">
         <v>46226</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1332,7 +1331,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Factura C monotributo Sol · PELESSON ALDO OSCAR</t>
+          <t>Factura C PELESSON</t>
         </is>
       </c>
       <c r="F2" s="20" t="n">
@@ -1340,7 +1339,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>COBRADO → Reserva Chris</t>
+          <t>COBRADO → Chris</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1349,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B3" s="35" t="n">
+      <c r="B3" s="25" t="n">
         <v>46157</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1365,17 +1364,13 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
+          <t>Transferencia PELESSON</t>
         </is>
       </c>
       <c r="F3" s="20" t="n">
         <v>5000000</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Cobro MP histórico</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1383,7 +1378,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B4" s="35" t="n">
+      <c r="B4" s="25" t="n">
         <v>46185</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1398,17 +1393,13 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Transferencia recibida PELESSON ALDO OSCAR</t>
+          <t>Transferencia PELESSON</t>
         </is>
       </c>
       <c r="F4" s="20" t="n">
         <v>4750000</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Cobro MP histórico</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1416,7 +1407,7 @@
           <t>COBRO</t>
         </is>
       </c>
-      <c r="B5" s="35" t="n">
+      <c r="B5" s="25" t="n">
         <v>46226</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1426,139 +1417,124 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Cobro MP Factura C 00001-00000027</t>
+          <t>Cobro Factura C 00001-00000027</t>
         </is>
       </c>
       <c r="F5" s="20" t="n">
         <v>4900000</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>→ Reserva Chris</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RESERVA</t>
-        </is>
-      </c>
-      <c r="B6" s="35" t="n">
-        <v>46158</v>
+          <t>PAGO_A_RESERVA</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n">
+        <v>46228</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mayo</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>158758469069</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Dinero reservado Chris</t>
+          <t>Pago Sol a la reserva</t>
         </is>
       </c>
       <c r="F6" s="20" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Ruteo cobro 15-may</t>
-        </is>
-      </c>
+        <v>2000000</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>RESERVA</t>
-        </is>
-      </c>
-      <c r="B7" s="35" t="n">
-        <v>46185</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Junio</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>163024353651</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Dinero reservado Chris</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>4500000</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Ruteo parcial 12-jun</t>
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>PAGO_A_RESERVA</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Julio</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="26" t="inlineStr">
+        <is>
+          <t>Pago Sol a la reserva (saldo deuda)</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="n">
+        <v>1510000</v>
+      </c>
+      <c r="G7" s="26" t="inlineStr">
+        <is>
+          <t>SALDA DEUDA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RESERVA</t>
-        </is>
-      </c>
-      <c r="B8" s="35" t="n">
-        <v>46226</v>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>46183</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Julio</t>
+          <t>Junio</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>163418872656</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dinero reservado Chris</t>
+          <t>Dinero retirado Chris</t>
         </is>
       </c>
       <c r="F8" s="20" t="n">
-        <v>4900000</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Factura → Chris</t>
-        </is>
-      </c>
+        <v>500000</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PAGO_DEUDA</t>
-        </is>
-      </c>
-      <c r="B9" s="35" t="n">
-        <v>46228</v>
+          <t>RETIRO</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>46193</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>165013974648</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pago a Reserva Chris</t>
+          <t>Dinero retirado Chris</t>
         </is>
       </c>
       <c r="F9" s="20" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Confirmación Sol</t>
-        </is>
-      </c>
+        <v>20000</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1566,17 +1542,17 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B10" s="35" t="n">
-        <v>46183</v>
+      <c r="B10" s="25" t="n">
+        <v>46196</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Junio</t>
+          <t>Julio</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>163418872656</t>
+          <t>165530199038</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1585,13 +1561,9 @@
         </is>
       </c>
       <c r="F10" s="20" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Retiro Junio</t>
-        </is>
-      </c>
+        <v>150000</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1599,8 +1571,8 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B11" s="35" t="n">
-        <v>46193</v>
+      <c r="B11" s="25" t="n">
+        <v>46198</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1609,7 +1581,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>165013974648</t>
+          <t>165824407784</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1618,13 +1590,9 @@
         </is>
       </c>
       <c r="F11" s="20" t="n">
-        <v>20000</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>extracto 20-jun</t>
-        </is>
-      </c>
+        <v>170000</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1632,197 +1600,122 @@
           <t>RETIRO</t>
         </is>
       </c>
-      <c r="B12" s="35" t="n">
-        <v>46196</v>
+      <c r="B12" s="25" t="n">
+        <v>46228</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>165530199038</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>Dinero retirado Chris</t>
         </is>
       </c>
       <c r="F12" s="20" t="n">
-        <v>150000</v>
+        <v>500000</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>extracto 23-jun</t>
+          <t>bajar reserva</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B13" s="35" t="n">
-        <v>46198</v>
+          <t>DEUDA_INICIAL</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="n">
+        <v>46226</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>165824407784</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Dinero retirado Chris</t>
+          <t>Deuda original Sol a Chris</t>
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>170000</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>consolidado 170000</t>
-        </is>
-      </c>
+        <v>3510000</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
-        <is>
-          <t>RETIRO</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="n">
-        <v>46228</v>
-      </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>DEUDA_RESERVA_CHRIS</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="28" t="inlineStr">
-        <is>
-          <t>Dinero retirado Chris</t>
-        </is>
-      </c>
-      <c r="F14" s="30" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G14" s="28" t="inlineStr">
-        <is>
-          <t>Bajar reserva · Sol</t>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>Deuda restante (SALDADA)</t>
+        </is>
+      </c>
+      <c r="F14" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="29" t="inlineStr">
+        <is>
+          <t>3510000-2000000-1510000</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SALDO_CAJA</t>
+          <t>SALDO_CHRIS_ACTUAL</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Julio</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Saldo caja UDESA consolidado</t>
+          <t>Saldo actual Reserva Chris</t>
         </is>
       </c>
       <c r="F15" s="20" t="n">
         <v>13310000</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>14650000-1340000</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SALDO_CHRIS_ACTUAL</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="n">
-        <v>46228</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Julio</t>
+          <t>SALDO_CAJA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Saldo actual Reserva Chris</t>
+          <t>Saldo caja UDESA</t>
         </is>
       </c>
       <c r="F16" s="20" t="n">
-        <v>11800000</v>
+        <v>13310000</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10300000+2000000-500000</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="28" t="inlineStr">
-        <is>
-          <t>DEUDA_RESERVA_CHRIS</t>
-        </is>
-      </c>
-      <c r="B17" s="36" t="n">
-        <v>46228</v>
-      </c>
-      <c r="C17" s="28" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="D17" s="28" t="n"/>
-      <c r="E17" s="28" t="inlineStr">
-        <is>
-          <t>Deuda restante Sol a Reserva Chris (le debo)</t>
-        </is>
-      </c>
-      <c r="F17" s="30" t="n">
-        <v>1510000</v>
-      </c>
-      <c r="G17" s="28" t="inlineStr">
-        <is>
-          <t>3510000 - 2000000</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>DEUDA_INICIAL</t>
-        </is>
-      </c>
-      <c r="B18" s="35" t="n">
-        <v>46226</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Julio</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Deuda original Sol a Reserva Chris</t>
-        </is>
-      </c>
-      <c r="F18" s="20" t="n">
-        <v>3510000</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Indicación Sol</t>
+          <t>14650000-1340000</t>
         </is>
       </c>
     </row>

</xml_diff>